<commit_message>
modified:   outputs/TEX_output.xlsx 	new file:   outputs/cg_summary_500.csv 	new file:   outputs/hydro_500.csv 	new file:   outputs/stability_check_500.csv 	new file:   outputs/weights_500.csv
</commit_message>
<xml_diff>
--- a/outputs/TEX_output.xlsx
+++ b/outputs/TEX_output.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,19 +511,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="D3" t="n">
         <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>-500</v>
+        <v>-1000</v>
       </c>
       <c r="F3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -535,7 +535,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WEIGHTED KEEL (AFT)</t>
+          <t>MOTOR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -544,19 +544,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>250</v>
+        <v>145</v>
       </c>
       <c r="D4" t="n">
-        <v>-2</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
-        <v>-500</v>
+        <v>217.5</v>
       </c>
       <c r="F4" t="n">
-        <v>-7</v>
+        <v>-1.08</v>
       </c>
       <c r="G4" t="n">
-        <v>-1750</v>
+        <v>-156.6</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MOTOR</t>
+          <t>CONNING TOWER</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -577,19 +577,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>145</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="E5" t="n">
-        <v>217.5</v>
+        <v>140</v>
       </c>
       <c r="F5" t="n">
         <v>-1.08</v>
       </c>
       <c r="G5" t="n">
-        <v>-156.6</v>
+        <v>-43.2</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -601,28 +601,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CONNING TOWER</t>
+          <t>ELECTRONICS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CTR</t>
+          <t>PORT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>3.5</v>
+        <v>7.125</v>
       </c>
       <c r="E6" t="n">
-        <v>140</v>
+        <v>71.25</v>
       </c>
       <c r="F6" t="n">
         <v>-1.08</v>
       </c>
       <c r="G6" t="n">
-        <v>-43.2</v>
+        <v>-10.8</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -634,28 +634,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ELECTRONICS</t>
+          <t>BATTERY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PORT</t>
+          <t>STBD</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>20.85</v>
       </c>
       <c r="D7" t="n">
-        <v>7.125</v>
+        <v>0.583</v>
       </c>
       <c r="E7" t="n">
-        <v>71.25</v>
+        <v>12.15555</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.08</v>
+        <v>3.083</v>
       </c>
       <c r="G7" t="n">
-        <v>-10.8</v>
+        <v>64.28055000000001</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -667,7 +667,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BATTERY</t>
+          <t>GAS TANK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -676,19 +676,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.85</v>
+        <v>33.92</v>
       </c>
       <c r="D8" t="n">
         <v>0.583</v>
       </c>
       <c r="E8" t="n">
-        <v>12.15555</v>
+        <v>19.77536</v>
       </c>
       <c r="F8" t="n">
-        <v>3.083</v>
+        <v>3.833</v>
       </c>
       <c r="G8" t="n">
-        <v>64.28055000000001</v>
+        <v>130.01536</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -700,7 +700,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GAS TANK</t>
+          <t>DIVING PLANE FRONT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -709,19 +709,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>33.92</v>
+        <v>3.1</v>
       </c>
       <c r="D9" t="n">
-        <v>0.583</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>19.77536</v>
+        <v>3.1</v>
       </c>
       <c r="F9" t="n">
-        <v>3.833</v>
+        <v>7.5</v>
       </c>
       <c r="G9" t="n">
-        <v>130.01536</v>
+        <v>23.25</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -733,7 +733,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DIVING PLANE FRONT</t>
+          <t>DIVING PLANE BACK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -751,10 +751,10 @@
         <v>3.1</v>
       </c>
       <c r="F10" t="n">
-        <v>7.5</v>
+        <v>-7.5</v>
       </c>
       <c r="G10" t="n">
-        <v>23.25</v>
+        <v>-23.25</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -766,7 +766,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIVING PLANE BACK</t>
+          <t>RUDDER BACK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -784,10 +784,10 @@
         <v>3.1</v>
       </c>
       <c r="F11" t="n">
-        <v>-7.5</v>
+        <v>-8.542</v>
       </c>
       <c r="G11" t="n">
-        <v>-23.25</v>
+        <v>-26.4802</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -799,7 +799,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RUDDER BACK</t>
+          <t>RUDDER FRONT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -817,10 +817,10 @@
         <v>3.1</v>
       </c>
       <c r="F12" t="n">
-        <v>-8.542</v>
+        <v>8.583</v>
       </c>
       <c r="G12" t="n">
-        <v>-26.4802</v>
+        <v>26.6073</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -832,7 +832,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RUDDER FRONT</t>
+          <t>SERVO+BOX+OIL FRONT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -841,19 +841,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.1</v>
+        <v>20.1</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3.1</v>
+        <v>20.1</v>
       </c>
       <c r="F13" t="n">
-        <v>8.583</v>
+        <v>7.5</v>
       </c>
       <c r="G13" t="n">
-        <v>26.6073</v>
+        <v>150.75</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -865,7 +865,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SERVO+BOX+OIL FRONT</t>
+          <t>SERVO+BOX+OIL BACK</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -883,10 +883,10 @@
         <v>20.1</v>
       </c>
       <c r="F14" t="n">
-        <v>7.5</v>
+        <v>-7.5</v>
       </c>
       <c r="G14" t="n">
-        <v>150.75</v>
+        <v>-150.75</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -898,7 +898,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SERVO+BOX+OIL BACK</t>
+          <t>SERVO+BOX+OIL RUDDER FRONT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -916,10 +916,10 @@
         <v>20.1</v>
       </c>
       <c r="F15" t="n">
-        <v>-7.5</v>
+        <v>8.583</v>
       </c>
       <c r="G15" t="n">
-        <v>-150.75</v>
+        <v>172.5183</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -931,7 +931,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SERVO+BOX+OIL RUDDER FRONT</t>
+          <t>SERVO+BOX+OIL RUDDER BACK</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -949,48 +949,15 @@
         <v>20.1</v>
       </c>
       <c r="F16" t="n">
-        <v>8.583</v>
+        <v>-8.542</v>
       </c>
       <c r="G16" t="n">
-        <v>172.5183</v>
+        <v>-171.6942</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SERVO+BOX+OIL RUDDER BACK</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>STBD</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-8.542</v>
-      </c>
-      <c r="G17" t="n">
-        <v>-171.6942</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>